<commit_message>
new command to upload user
</commit_message>
<xml_diff>
--- a/src/laboratory/management/commands/Usuarios_por_laboratorio.xlsx
+++ b/src/laboratory/management/commands/Usuarios_por_laboratorio.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="269">
   <si>
     <t xml:space="preserve">Dirección de correo electrónico</t>
   </si>
@@ -172,7 +172,7 @@
     <t xml:space="preserve">allan.madrigal.mata@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">Asistencia Administrativa</t>
+    <t xml:space="preserve">Asistencia Administrativa Sarapiqui</t>
   </si>
   <si>
     <t xml:space="preserve">Sección Regional Huetar Norte y Caribe Campus Sarapiquí</t>
@@ -298,7 +298,7 @@
     <t xml:space="preserve">jose.sibaja.brenes@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">Laboratorio de Química de la Atmósfera (LAQAT-UNA)</t>
+    <t xml:space="preserve">Laboratorio de Química de la Atmósfera</t>
   </si>
   <si>
     <t xml:space="preserve">Stephanie Salas Alfaro</t>
@@ -337,7 +337,7 @@
     <t xml:space="preserve">alonso.calvo.araya@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">Director </t>
+    <t xml:space="preserve">Direccion</t>
   </si>
   <si>
     <t xml:space="preserve">Escuela de Ciencias Agrarias</t>
@@ -550,9 +550,6 @@
     <t xml:space="preserve">laqat@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">Laboratorio de Química de la Atmósfera</t>
-  </si>
-  <si>
     <t xml:space="preserve">Rosa Alfaro Solís</t>
   </si>
   <si>
@@ -601,7 +598,7 @@
     <t xml:space="preserve">irena.hilje.rodriguez@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">LABORATORIO DE BIOLOGÍA MOLECULAR</t>
+    <t xml:space="preserve">Biología Molecular</t>
   </si>
   <si>
     <t xml:space="preserve">IRENA HILJE RODRÍGUEZ</t>
@@ -649,7 +646,7 @@
     <t xml:space="preserve">gea.bonilla.duran@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">Laboratorio de Bioquímica</t>
+    <t xml:space="preserve">Laboratorio de Bioquímica y Biotecnología de Proteínas</t>
   </si>
   <si>
     <t xml:space="preserve">Gea Bonilla Durán</t>
@@ -733,7 +730,7 @@
     <t xml:space="preserve">wendy.sandoval.diaz@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">UNIDAD DE APOYO</t>
+    <t xml:space="preserve">Unidad de apoyo</t>
   </si>
   <si>
     <t xml:space="preserve">Luis Alberto Delgado Orozco</t>
@@ -826,7 +823,7 @@
     <t xml:space="preserve">isidro.calero.ocon@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">Laboratorio de Cultivo de Tejidos de Docencia </t>
+    <t xml:space="preserve">Cultivo de Tejidos (investigación)</t>
   </si>
   <si>
     <t xml:space="preserve">Isidro Calero Ocon </t>
@@ -842,9 +839,6 @@
   </si>
   <si>
     <t xml:space="preserve">Jefferson Aráuz Badilla</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Laboratorio de Cultivo de Tejidos Vegetales de Docencia.</t>
   </si>
   <si>
     <t xml:space="preserve">Isidro Calero Ocon</t>
@@ -2029,7 +2023,7 @@
         <v>155</v>
       </c>
       <c r="B30" s="8" t="s">
-        <v>156</v>
+        <v>72</v>
       </c>
       <c r="C30" s="9" t="s">
         <v>38</v>
@@ -2044,18 +2038,18 @@
         <v>74</v>
       </c>
       <c r="G30" s="7" t="s">
+        <v>156</v>
+      </c>
+      <c r="H30" s="7" t="s">
         <v>157</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>158</v>
       </c>
     </row>
     <row r="31" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
+        <v>158</v>
+      </c>
+      <c r="B31" s="9" t="s">
         <v>159</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>160</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>38</v>
@@ -2064,13 +2058,13 @@
         <v>39</v>
       </c>
       <c r="E31" s="7" t="s">
+        <v>160</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="G31" s="7" t="s">
         <v>161</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>162</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>52</v>
@@ -2078,10 +2072,10 @@
     </row>
     <row r="32" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>163</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>164</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>10</v>
@@ -2090,22 +2084,22 @@
         <v>11</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G32" s="7"/>
       <c r="H32" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="33" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
+        <v>162</v>
+      </c>
+      <c r="B33" s="11" t="s">
         <v>163</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>164</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>10</v>
@@ -2114,22 +2108,22 @@
         <v>11</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="G33" s="7"/>
       <c r="H33" s="7" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
     </row>
     <row r="34" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
+        <v>166</v>
+      </c>
+      <c r="B34" s="9" t="s">
         <v>167</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>38</v>
@@ -2138,24 +2132,24 @@
         <v>39</v>
       </c>
       <c r="E34" s="7" t="s">
+        <v>168</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="G34" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="F34" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="G34" s="7" t="s">
+      <c r="H34" s="7" t="s">
         <v>170</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
+        <v>171</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>172</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>173</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>86</v>
@@ -2164,72 +2158,72 @@
         <v>39</v>
       </c>
       <c r="E35" s="7" t="s">
+        <v>173</v>
+      </c>
+      <c r="F35" s="9" t="s">
         <v>174</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>175</v>
       </c>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
     </row>
     <row r="36" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B36" s="13" t="s">
         <v>176</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="C36" s="9" t="s">
         <v>177</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="D36" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E36" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E36" s="7" t="s">
+      <c r="F36" s="9" t="s">
+        <v>175</v>
+      </c>
+      <c r="G36" s="7" t="s">
         <v>179</v>
       </c>
-      <c r="F36" s="9" t="s">
-        <v>176</v>
-      </c>
-      <c r="G36" s="7" t="s">
+      <c r="H36" s="7" t="s">
         <v>180</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="37" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
+        <v>181</v>
+      </c>
+      <c r="B37" s="9" t="s">
         <v>182</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="C37" s="9" t="s">
+        <v>177</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E37" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="C37" s="9" t="s">
-        <v>178</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E37" s="7" t="s">
+      <c r="F37" s="9" t="s">
         <v>184</v>
       </c>
-      <c r="F37" s="9" t="s">
+      <c r="G37" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="G37" s="7" t="s">
+      <c r="H37" s="7" t="s">
         <v>186</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="38" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
+        <v>187</v>
+      </c>
+      <c r="B38" s="15" t="s">
         <v>188</v>
-      </c>
-      <c r="B38" s="15" t="s">
-        <v>189</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>38</v>
@@ -2238,10 +2232,10 @@
         <v>39</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="H38" s="7" t="s">
         <v>52</v>
@@ -2249,48 +2243,48 @@
     </row>
     <row r="39" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
+        <v>190</v>
+      </c>
+      <c r="B39" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="C39" s="9" t="s">
         <v>192</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="D39" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E39" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="D39" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E39" s="7" t="s">
+      <c r="F39" s="9" t="s">
+        <v>190</v>
+      </c>
+      <c r="G39" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="F39" s="9" t="s">
-        <v>191</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>195</v>
-      </c>
       <c r="H39" s="7" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="40" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
+        <v>195</v>
+      </c>
+      <c r="B40" s="13" t="s">
         <v>196</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="C40" s="9" t="s">
         <v>197</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>198</v>
       </c>
       <c r="D40" s="9" t="s">
         <v>114</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G40" s="7" t="s">
         <v>115</v>
@@ -2301,22 +2295,22 @@
     </row>
     <row r="41" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>114</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G41" s="7" t="s">
         <v>115</v>
@@ -2327,22 +2321,22 @@
     </row>
     <row r="42" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="16" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>114</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="G42" s="7" t="s">
         <v>115</v>
@@ -2353,10 +2347,10 @@
     </row>
     <row r="43" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
+        <v>201</v>
+      </c>
+      <c r="B43" s="9" t="s">
         <v>202</v>
-      </c>
-      <c r="B43" s="9" t="s">
-        <v>203</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>10</v>
@@ -2365,72 +2359,72 @@
         <v>11</v>
       </c>
       <c r="E43" s="7" t="s">
+        <v>203</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>201</v>
+      </c>
+      <c r="G43" s="7" t="s">
         <v>204</v>
       </c>
-      <c r="F43" s="9" t="s">
-        <v>202</v>
-      </c>
-      <c r="G43" s="7" t="s">
+      <c r="H43" s="7" t="s">
         <v>205</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>206</v>
       </c>
     </row>
     <row r="44" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
+        <v>206</v>
+      </c>
+      <c r="B44" s="9" t="s">
         <v>207</v>
       </c>
-      <c r="B44" s="9" t="s">
+      <c r="C44" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E44" s="7" t="s">
         <v>208</v>
       </c>
-      <c r="C44" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>209</v>
-      </c>
       <c r="F44" s="9" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="G44" s="7"/>
       <c r="H44" s="7"/>
     </row>
     <row r="45" s="1" customFormat="true" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
+        <v>209</v>
+      </c>
+      <c r="B45" s="9" t="s">
         <v>210</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="C45" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E45" s="7" t="s">
         <v>211</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E45" s="7" t="s">
+      <c r="F45" s="9" t="s">
         <v>212</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="G45" s="7" t="s">
         <v>213</v>
       </c>
-      <c r="G45" s="7" t="s">
+      <c r="H45" s="7" t="s">
         <v>214</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>215</v>
       </c>
     </row>
     <row r="46" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
+        <v>215</v>
+      </c>
+      <c r="B46" s="9" t="s">
         <v>216</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>217</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>47</v>
@@ -2439,20 +2433,20 @@
         <v>39</v>
       </c>
       <c r="E46" s="7" t="s">
+        <v>217</v>
+      </c>
+      <c r="F46" s="9" t="s">
         <v>218</v>
-      </c>
-      <c r="F46" s="9" t="s">
-        <v>219</v>
       </c>
       <c r="G46" s="7"/>
       <c r="H46" s="7"/>
     </row>
     <row r="47" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
+        <v>219</v>
+      </c>
+      <c r="B47" s="13" t="s">
         <v>220</v>
-      </c>
-      <c r="B47" s="13" t="s">
-        <v>221</v>
       </c>
       <c r="C47" s="9" t="s">
         <v>38</v>
@@ -2461,76 +2455,76 @@
         <v>39</v>
       </c>
       <c r="E47" s="7" t="s">
+        <v>221</v>
+      </c>
+      <c r="F47" s="9" t="s">
         <v>222</v>
       </c>
-      <c r="F47" s="9" t="s">
-        <v>223</v>
-      </c>
       <c r="G47" s="7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
+        <v>223</v>
+      </c>
+      <c r="B48" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="B48" s="9" t="s">
+      <c r="C48" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="D48" s="9" t="s">
         <v>225</v>
       </c>
-      <c r="C48" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="D48" s="9" t="s">
+      <c r="E48" s="7" t="s">
         <v>226</v>
       </c>
-      <c r="E48" s="7" t="s">
+      <c r="F48" s="9" t="s">
         <v>227</v>
       </c>
-      <c r="F48" s="9" t="s">
+      <c r="G48" s="7" t="s">
         <v>228</v>
       </c>
-      <c r="G48" s="7" t="s">
-        <v>229</v>
-      </c>
       <c r="H48" s="7" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
+        <v>229</v>
+      </c>
+      <c r="B49" s="15" t="s">
         <v>230</v>
       </c>
-      <c r="B49" s="15" t="s">
+      <c r="C49" s="9" t="s">
         <v>231</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="D49" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E49" s="7" t="s">
         <v>232</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E49" s="7" t="s">
-        <v>233</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>62</v>
       </c>
       <c r="G49" s="7" t="s">
+        <v>233</v>
+      </c>
+      <c r="H49" s="7" t="s">
         <v>234</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>235</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
+        <v>235</v>
+      </c>
+      <c r="B50" s="9" t="s">
         <v>236</v>
-      </c>
-      <c r="B50" s="9" t="s">
-        <v>237</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>86</v>
@@ -2539,24 +2533,24 @@
         <v>39</v>
       </c>
       <c r="E50" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="F50" s="9" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="G50" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="H50" s="7" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
     </row>
     <row r="51" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="B51" s="9" t="s">
         <v>239</v>
-      </c>
-      <c r="B51" s="9" t="s">
-        <v>240</v>
       </c>
       <c r="C51" s="9" t="s">
         <v>86</v>
@@ -2565,16 +2559,16 @@
         <v>39</v>
       </c>
       <c r="E51" s="7" t="s">
+        <v>240</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>238</v>
+      </c>
+      <c r="G51" s="7" t="s">
         <v>241</v>
       </c>
-      <c r="F51" s="9" t="s">
-        <v>239</v>
-      </c>
-      <c r="G51" s="7" t="s">
+      <c r="H51" s="7" t="s">
         <v>242</v>
-      </c>
-      <c r="H51" s="7" t="s">
-        <v>243</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2582,7 +2576,7 @@
         <v>61</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="C52" s="9" t="s">
         <v>10</v>
@@ -2591,7 +2585,7 @@
         <v>11</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>57</v>
@@ -2600,15 +2594,15 @@
         <v>60</v>
       </c>
       <c r="H52" s="7" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="B53" s="15" t="s">
         <v>247</v>
-      </c>
-      <c r="B53" s="15" t="s">
-        <v>248</v>
       </c>
       <c r="C53" s="9" t="s">
         <v>86</v>
@@ -2617,19 +2611,19 @@
         <v>39</v>
       </c>
       <c r="E53" s="7" t="s">
+        <v>248</v>
+      </c>
+      <c r="F53" s="9" t="s">
         <v>249</v>
-      </c>
-      <c r="F53" s="9" t="s">
-        <v>250</v>
       </c>
       <c r="H53" s="7"/>
     </row>
     <row r="54" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
+        <v>250</v>
+      </c>
+      <c r="B54" s="9" t="s">
         <v>251</v>
-      </c>
-      <c r="B54" s="9" t="s">
-        <v>252</v>
       </c>
       <c r="C54" s="9" t="s">
         <v>86</v>
@@ -2638,20 +2632,20 @@
         <v>39</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>253</v>
+        <v>252</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="G54" s="7"/>
       <c r="H54" s="7"/>
     </row>
     <row r="55" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
+        <v>246</v>
+      </c>
+      <c r="B55" s="17" t="s">
         <v>247</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>254</v>
       </c>
       <c r="C55" s="9" t="s">
         <v>86</v>
@@ -2660,76 +2654,76 @@
         <v>39</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>255</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E56" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="B56" s="9" t="s">
+      <c r="F56" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="G56" s="7" t="s">
         <v>257</v>
       </c>
-      <c r="C56" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E56" s="7" t="s">
+      <c r="H56" s="7" t="s">
         <v>258</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="G56" s="7" t="s">
-        <v>259</v>
-      </c>
-      <c r="H56" s="7" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
+        <v>254</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>259</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>192</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E57" s="7" t="s">
         <v>256</v>
       </c>
-      <c r="B57" s="9" t="s">
-        <v>261</v>
-      </c>
-      <c r="C57" s="9" t="s">
-        <v>193</v>
-      </c>
-      <c r="D57" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E57" s="7" t="s">
+      <c r="F57" s="9" t="s">
+        <v>254</v>
+      </c>
+      <c r="G57" s="7" t="s">
+        <v>257</v>
+      </c>
+      <c r="H57" s="7" t="s">
         <v>258</v>
-      </c>
-      <c r="F57" s="9" t="s">
-        <v>256</v>
-      </c>
-      <c r="G57" s="7" t="s">
-        <v>259</v>
-      </c>
-      <c r="H57" s="7" t="s">
-        <v>260</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B58" s="17" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C58" s="9" t="s">
         <v>86</v>
@@ -2738,42 +2732,42 @@
         <v>39</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="H58" s="7" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
+        <v>263</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>264</v>
+      </c>
+      <c r="C59" s="9" t="s">
         <v>265</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="D59" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E59" s="7" t="s">
         <v>266</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="F59" s="9" t="s">
+        <v>263</v>
+      </c>
+      <c r="G59" s="7" t="s">
         <v>267</v>
       </c>
-      <c r="D59" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E59" s="7" t="s">
+      <c r="H59" s="7" t="s">
         <v>268</v>
-      </c>
-      <c r="F59" s="9" t="s">
-        <v>265</v>
-      </c>
-      <c r="G59" s="7" t="s">
-        <v>269</v>
-      </c>
-      <c r="H59" s="7" t="s">
-        <v>270</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Update command to upload users
</commit_message>
<xml_diff>
--- a/src/laboratory/management/commands/Usuarios_por_laboratorio.xlsx
+++ b/src/laboratory/management/commands/Usuarios_por_laboratorio.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="447" uniqueCount="269">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="266">
   <si>
     <t xml:space="preserve">Dirección de correo electrónico</t>
   </si>
@@ -526,9 +526,6 @@
     <t xml:space="preserve">ronald.molina.ulate@una.cr</t>
   </si>
   <si>
-    <t xml:space="preserve">.</t>
-  </si>
-  <si>
     <t xml:space="preserve">alejandro.alfaro.alarcon@una.cr</t>
   </si>
   <si>
@@ -793,9 +790,6 @@
     <t xml:space="preserve">Laboratorio de Fitopatología Investigación</t>
   </si>
   <si>
-    <t xml:space="preserve">--</t>
-  </si>
-  <si>
     <t xml:space="preserve">roy.artavia.carmona@una.cr</t>
   </si>
   <si>
@@ -815,9 +809,6 @@
   </si>
   <si>
     <t xml:space="preserve">Alejandra Calderón Hernández</t>
-  </si>
-  <si>
-    <t xml:space="preserve">monica.narvaez.ruano</t>
   </si>
   <si>
     <t xml:space="preserve">isidro.calero.ocon@una.cr</t>
@@ -1988,16 +1979,14 @@
         <v>88</v>
       </c>
       <c r="G28" s="7"/>
-      <c r="H28" s="7" t="s">
-        <v>148</v>
-      </c>
+      <c r="H28" s="7"/>
     </row>
     <row r="29" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="B29" s="12" t="s">
         <v>149</v>
-      </c>
-      <c r="B29" s="12" t="s">
-        <v>150</v>
       </c>
       <c r="C29" s="9" t="s">
         <v>10</v>
@@ -2006,21 +1995,21 @@
         <v>11</v>
       </c>
       <c r="E29" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="F29" s="9" t="s">
         <v>151</v>
       </c>
-      <c r="F29" s="9" t="s">
+      <c r="G29" s="7" t="s">
         <v>152</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="H29" s="7" t="s">
         <v>153</v>
-      </c>
-      <c r="H29" s="7" t="s">
-        <v>154</v>
       </c>
     </row>
     <row r="30" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="7" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B30" s="8" t="s">
         <v>72</v>
@@ -2038,18 +2027,18 @@
         <v>74</v>
       </c>
       <c r="G30" s="7" t="s">
+        <v>155</v>
+      </c>
+      <c r="H30" s="7" t="s">
         <v>156</v>
-      </c>
-      <c r="H30" s="7" t="s">
-        <v>157</v>
       </c>
     </row>
     <row r="31" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A31" s="7" t="s">
+        <v>157</v>
+      </c>
+      <c r="B31" s="9" t="s">
         <v>158</v>
-      </c>
-      <c r="B31" s="9" t="s">
-        <v>159</v>
       </c>
       <c r="C31" s="9" t="s">
         <v>38</v>
@@ -2058,13 +2047,13 @@
         <v>39</v>
       </c>
       <c r="E31" s="7" t="s">
+        <v>159</v>
+      </c>
+      <c r="F31" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="G31" s="7" t="s">
         <v>160</v>
-      </c>
-      <c r="F31" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>161</v>
       </c>
       <c r="H31" s="7" t="s">
         <v>52</v>
@@ -2072,10 +2061,10 @@
     </row>
     <row r="32" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A32" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B32" s="11" t="s">
         <v>162</v>
-      </c>
-      <c r="B32" s="11" t="s">
-        <v>163</v>
       </c>
       <c r="C32" s="9" t="s">
         <v>10</v>
@@ -2084,22 +2073,22 @@
         <v>11</v>
       </c>
       <c r="E32" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F32" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G32" s="7"/>
       <c r="H32" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="33" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A33" s="7" t="s">
+        <v>161</v>
+      </c>
+      <c r="B33" s="11" t="s">
         <v>162</v>
-      </c>
-      <c r="B33" s="11" t="s">
-        <v>163</v>
       </c>
       <c r="C33" s="9" t="s">
         <v>10</v>
@@ -2108,22 +2097,22 @@
         <v>11</v>
       </c>
       <c r="E33" s="7" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F33" s="9" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="G33" s="7"/>
       <c r="H33" s="7" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
     </row>
     <row r="34" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A34" s="7" t="s">
+        <v>165</v>
+      </c>
+      <c r="B34" s="9" t="s">
         <v>166</v>
-      </c>
-      <c r="B34" s="9" t="s">
-        <v>167</v>
       </c>
       <c r="C34" s="9" t="s">
         <v>38</v>
@@ -2132,24 +2121,24 @@
         <v>39</v>
       </c>
       <c r="E34" s="7" t="s">
+        <v>167</v>
+      </c>
+      <c r="F34" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="G34" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="F34" s="9" t="s">
-        <v>166</v>
-      </c>
-      <c r="G34" s="7" t="s">
+      <c r="H34" s="7" t="s">
         <v>169</v>
-      </c>
-      <c r="H34" s="7" t="s">
-        <v>170</v>
       </c>
     </row>
     <row r="35" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A35" s="7" t="s">
+        <v>170</v>
+      </c>
+      <c r="B35" s="15" t="s">
         <v>171</v>
-      </c>
-      <c r="B35" s="15" t="s">
-        <v>172</v>
       </c>
       <c r="C35" s="9" t="s">
         <v>86</v>
@@ -2158,72 +2147,72 @@
         <v>39</v>
       </c>
       <c r="E35" s="7" t="s">
+        <v>172</v>
+      </c>
+      <c r="F35" s="9" t="s">
         <v>173</v>
-      </c>
-      <c r="F35" s="9" t="s">
-        <v>174</v>
       </c>
       <c r="G35" s="7"/>
       <c r="H35" s="7"/>
     </row>
     <row r="36" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A36" s="7" t="s">
+        <v>174</v>
+      </c>
+      <c r="B36" s="13" t="s">
         <v>175</v>
       </c>
-      <c r="B36" s="13" t="s">
+      <c r="C36" s="9" t="s">
         <v>176</v>
       </c>
-      <c r="C36" s="9" t="s">
+      <c r="D36" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E36" s="7" t="s">
         <v>177</v>
       </c>
-      <c r="D36" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E36" s="7" t="s">
+      <c r="F36" s="9" t="s">
+        <v>174</v>
+      </c>
+      <c r="G36" s="7" t="s">
         <v>178</v>
       </c>
-      <c r="F36" s="9" t="s">
-        <v>175</v>
-      </c>
-      <c r="G36" s="7" t="s">
+      <c r="H36" s="7" t="s">
         <v>179</v>
-      </c>
-      <c r="H36" s="7" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="37" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A37" s="7" t="s">
+        <v>180</v>
+      </c>
+      <c r="B37" s="9" t="s">
         <v>181</v>
       </c>
-      <c r="B37" s="9" t="s">
+      <c r="C37" s="9" t="s">
+        <v>176</v>
+      </c>
+      <c r="D37" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E37" s="7" t="s">
         <v>182</v>
       </c>
-      <c r="C37" s="9" t="s">
-        <v>177</v>
-      </c>
-      <c r="D37" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E37" s="7" t="s">
+      <c r="F37" s="9" t="s">
         <v>183</v>
       </c>
-      <c r="F37" s="9" t="s">
+      <c r="G37" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="G37" s="7" t="s">
+      <c r="H37" s="7" t="s">
         <v>185</v>
-      </c>
-      <c r="H37" s="7" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="38" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A38" s="7" t="s">
+        <v>186</v>
+      </c>
+      <c r="B38" s="15" t="s">
         <v>187</v>
-      </c>
-      <c r="B38" s="15" t="s">
-        <v>188</v>
       </c>
       <c r="C38" s="9" t="s">
         <v>38</v>
@@ -2232,10 +2221,10 @@
         <v>39</v>
       </c>
       <c r="E38" s="7" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="F38" s="9" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="H38" s="7" t="s">
         <v>52</v>
@@ -2243,48 +2232,48 @@
     </row>
     <row r="39" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A39" s="7" t="s">
+        <v>189</v>
+      </c>
+      <c r="B39" s="9" t="s">
         <v>190</v>
       </c>
-      <c r="B39" s="9" t="s">
+      <c r="C39" s="9" t="s">
         <v>191</v>
       </c>
-      <c r="C39" s="9" t="s">
+      <c r="D39" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E39" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="D39" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E39" s="7" t="s">
+      <c r="F39" s="9" t="s">
+        <v>189</v>
+      </c>
+      <c r="G39" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="F39" s="9" t="s">
-        <v>190</v>
-      </c>
-      <c r="G39" s="7" t="s">
-        <v>194</v>
-      </c>
       <c r="H39" s="7" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="40" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A40" s="16" t="s">
+        <v>194</v>
+      </c>
+      <c r="B40" s="13" t="s">
         <v>195</v>
       </c>
-      <c r="B40" s="13" t="s">
+      <c r="C40" s="9" t="s">
         <v>196</v>
-      </c>
-      <c r="C40" s="9" t="s">
-        <v>197</v>
       </c>
       <c r="D40" s="9" t="s">
         <v>114</v>
       </c>
       <c r="E40" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F40" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G40" s="7" t="s">
         <v>115</v>
@@ -2295,22 +2284,22 @@
     </row>
     <row r="41" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A41" s="16" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B41" s="13" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="C41" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D41" s="9" t="s">
         <v>114</v>
       </c>
       <c r="E41" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F41" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G41" s="7" t="s">
         <v>115</v>
@@ -2321,22 +2310,22 @@
     </row>
     <row r="42" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A42" s="16" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B42" s="13" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="C42" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="D42" s="9" t="s">
         <v>114</v>
       </c>
       <c r="E42" s="7" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="F42" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="G42" s="7" t="s">
         <v>115</v>
@@ -2347,10 +2336,10 @@
     </row>
     <row r="43" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A43" s="7" t="s">
+        <v>200</v>
+      </c>
+      <c r="B43" s="9" t="s">
         <v>201</v>
-      </c>
-      <c r="B43" s="9" t="s">
-        <v>202</v>
       </c>
       <c r="C43" s="9" t="s">
         <v>10</v>
@@ -2359,72 +2348,72 @@
         <v>11</v>
       </c>
       <c r="E43" s="7" t="s">
+        <v>202</v>
+      </c>
+      <c r="F43" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="G43" s="7" t="s">
         <v>203</v>
       </c>
-      <c r="F43" s="9" t="s">
-        <v>201</v>
-      </c>
-      <c r="G43" s="7" t="s">
+      <c r="H43" s="7" t="s">
         <v>204</v>
-      </c>
-      <c r="H43" s="7" t="s">
-        <v>205</v>
       </c>
     </row>
     <row r="44" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A44" s="7" t="s">
+        <v>205</v>
+      </c>
+      <c r="B44" s="9" t="s">
         <v>206</v>
       </c>
-      <c r="B44" s="9" t="s">
+      <c r="C44" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="D44" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E44" s="7" t="s">
         <v>207</v>
       </c>
-      <c r="C44" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="D44" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E44" s="7" t="s">
-        <v>208</v>
-      </c>
       <c r="F44" s="9" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="G44" s="7"/>
       <c r="H44" s="7"/>
     </row>
     <row r="45" s="1" customFormat="true" ht="35.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A45" s="7" t="s">
+        <v>208</v>
+      </c>
+      <c r="B45" s="9" t="s">
         <v>209</v>
       </c>
-      <c r="B45" s="9" t="s">
+      <c r="C45" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="D45" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E45" s="7" t="s">
         <v>210</v>
       </c>
-      <c r="C45" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="D45" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E45" s="7" t="s">
+      <c r="F45" s="9" t="s">
         <v>211</v>
       </c>
-      <c r="F45" s="9" t="s">
+      <c r="G45" s="7" t="s">
         <v>212</v>
       </c>
-      <c r="G45" s="7" t="s">
+      <c r="H45" s="7" t="s">
         <v>213</v>
-      </c>
-      <c r="H45" s="7" t="s">
-        <v>214</v>
       </c>
     </row>
     <row r="46" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A46" s="7" t="s">
+        <v>214</v>
+      </c>
+      <c r="B46" s="9" t="s">
         <v>215</v>
-      </c>
-      <c r="B46" s="9" t="s">
-        <v>216</v>
       </c>
       <c r="C46" s="9" t="s">
         <v>47</v>
@@ -2433,20 +2422,20 @@
         <v>39</v>
       </c>
       <c r="E46" s="7" t="s">
+        <v>216</v>
+      </c>
+      <c r="F46" s="9" t="s">
         <v>217</v>
-      </c>
-      <c r="F46" s="9" t="s">
-        <v>218</v>
       </c>
       <c r="G46" s="7"/>
       <c r="H46" s="7"/>
     </row>
     <row r="47" s="1" customFormat="true" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A47" s="7" t="s">
+        <v>218</v>
+      </c>
+      <c r="B47" s="13" t="s">
         <v>219</v>
-      </c>
-      <c r="B47" s="13" t="s">
-        <v>220</v>
       </c>
       <c r="C47" s="9" t="s">
         <v>38</v>
@@ -2455,76 +2444,76 @@
         <v>39</v>
       </c>
       <c r="E47" s="7" t="s">
+        <v>220</v>
+      </c>
+      <c r="F47" s="9" t="s">
         <v>221</v>
       </c>
-      <c r="F47" s="9" t="s">
-        <v>222</v>
-      </c>
       <c r="G47" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="H47" s="7" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
     </row>
     <row r="48" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A48" s="7" t="s">
+        <v>222</v>
+      </c>
+      <c r="B48" s="9" t="s">
         <v>223</v>
       </c>
-      <c r="B48" s="9" t="s">
+      <c r="C48" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="D48" s="9" t="s">
         <v>224</v>
       </c>
-      <c r="C48" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="D48" s="9" t="s">
+      <c r="E48" s="7" t="s">
         <v>225</v>
       </c>
-      <c r="E48" s="7" t="s">
+      <c r="F48" s="9" t="s">
         <v>226</v>
       </c>
-      <c r="F48" s="9" t="s">
+      <c r="G48" s="7" t="s">
         <v>227</v>
       </c>
-      <c r="G48" s="7" t="s">
-        <v>228</v>
-      </c>
       <c r="H48" s="7" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
     </row>
     <row r="49" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A49" s="7" t="s">
+        <v>228</v>
+      </c>
+      <c r="B49" s="15" t="s">
         <v>229</v>
       </c>
-      <c r="B49" s="15" t="s">
+      <c r="C49" s="9" t="s">
         <v>230</v>
       </c>
-      <c r="C49" s="9" t="s">
+      <c r="D49" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E49" s="7" t="s">
         <v>231</v>
-      </c>
-      <c r="D49" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E49" s="7" t="s">
-        <v>232</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>62</v>
       </c>
       <c r="G49" s="7" t="s">
+        <v>232</v>
+      </c>
+      <c r="H49" s="7" t="s">
         <v>233</v>
-      </c>
-      <c r="H49" s="7" t="s">
-        <v>234</v>
       </c>
     </row>
     <row r="50" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A50" s="7" t="s">
+        <v>234</v>
+      </c>
+      <c r="B50" s="9" t="s">
         <v>235</v>
-      </c>
-      <c r="B50" s="9" t="s">
-        <v>236</v>
       </c>
       <c r="C50" s="9" t="s">
         <v>86</v>
@@ -2532,25 +2521,19 @@
       <c r="D50" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="E50" s="7" t="s">
-        <v>237</v>
-      </c>
+      <c r="E50" s="7"/>
       <c r="F50" s="9" t="s">
-        <v>235</v>
-      </c>
-      <c r="G50" s="7" t="s">
-        <v>237</v>
-      </c>
-      <c r="H50" s="7" t="s">
-        <v>237</v>
-      </c>
+        <v>234</v>
+      </c>
+      <c r="G50" s="7"/>
+      <c r="H50" s="7"/>
     </row>
     <row r="51" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A51" s="7" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B51" s="9" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="C51" s="9" t="s">
         <v>86</v>
@@ -2559,16 +2542,16 @@
         <v>39</v>
       </c>
       <c r="E51" s="7" t="s">
+        <v>238</v>
+      </c>
+      <c r="F51" s="9" t="s">
+        <v>236</v>
+      </c>
+      <c r="G51" s="7" t="s">
+        <v>239</v>
+      </c>
+      <c r="H51" s="7" t="s">
         <v>240</v>
-      </c>
-      <c r="F51" s="9" t="s">
-        <v>238</v>
-      </c>
-      <c r="G51" s="7" t="s">
-        <v>241</v>
-      </c>
-      <c r="H51" s="7" t="s">
-        <v>242</v>
       </c>
     </row>
     <row r="52" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2576,7 +2559,7 @@
         <v>61</v>
       </c>
       <c r="B52" s="9" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="C52" s="9" t="s">
         <v>10</v>
@@ -2585,7 +2568,7 @@
         <v>11</v>
       </c>
       <c r="E52" s="7" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
       <c r="F52" s="9" t="s">
         <v>57</v>
@@ -2594,15 +2577,15 @@
         <v>60</v>
       </c>
       <c r="H52" s="7" t="s">
-        <v>245</v>
+        <v>61</v>
       </c>
     </row>
     <row r="53" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A53" s="7" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B53" s="15" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C53" s="9" t="s">
         <v>86</v>
@@ -2611,19 +2594,19 @@
         <v>39</v>
       </c>
       <c r="E53" s="7" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="F53" s="9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="H53" s="7"/>
     </row>
     <row r="54" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A54" s="7" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="B54" s="9" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="C54" s="9" t="s">
         <v>86</v>
@@ -2632,20 +2615,20 @@
         <v>39</v>
       </c>
       <c r="E54" s="7" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="F54" s="9" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="G54" s="7"/>
       <c r="H54" s="7"/>
     </row>
     <row r="55" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A55" s="7" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B55" s="17" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="C55" s="9" t="s">
         <v>86</v>
@@ -2654,76 +2637,76 @@
         <v>39</v>
       </c>
       <c r="E55" s="7" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="F55" s="9" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="G55" s="7" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="H55" s="7" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
     </row>
     <row r="56" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A56" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="B56" s="9" t="s">
+        <v>252</v>
+      </c>
+      <c r="C56" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="D56" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E56" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="F56" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="G56" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="B56" s="9" t="s">
+      <c r="H56" s="7" t="s">
         <v>255</v>
-      </c>
-      <c r="C56" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="D56" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E56" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="F56" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="G56" s="7" t="s">
-        <v>257</v>
-      </c>
-      <c r="H56" s="7" t="s">
-        <v>258</v>
       </c>
     </row>
     <row r="57" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A57" s="7" t="s">
+        <v>251</v>
+      </c>
+      <c r="B57" s="9" t="s">
+        <v>256</v>
+      </c>
+      <c r="C57" s="9" t="s">
+        <v>191</v>
+      </c>
+      <c r="D57" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E57" s="7" t="s">
+        <v>253</v>
+      </c>
+      <c r="F57" s="9" t="s">
+        <v>251</v>
+      </c>
+      <c r="G57" s="7" t="s">
         <v>254</v>
       </c>
-      <c r="B57" s="9" t="s">
-        <v>259</v>
-      </c>
-      <c r="C57" s="9" t="s">
-        <v>192</v>
-      </c>
-      <c r="D57" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E57" s="7" t="s">
-        <v>256</v>
-      </c>
-      <c r="F57" s="9" t="s">
-        <v>254</v>
-      </c>
-      <c r="G57" s="7" t="s">
-        <v>257</v>
-      </c>
       <c r="H57" s="7" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
     </row>
     <row r="58" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A58" s="7" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B58" s="17" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="C58" s="9" t="s">
         <v>86</v>
@@ -2732,42 +2715,42 @@
         <v>39</v>
       </c>
       <c r="E58" s="7" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="F58" s="9" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="G58" s="7" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="H58" s="7" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
     </row>
     <row r="59" customFormat="false" ht="22.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A59" s="7" t="s">
+        <v>260</v>
+      </c>
+      <c r="B59" s="9" t="s">
+        <v>261</v>
+      </c>
+      <c r="C59" s="9" t="s">
+        <v>262</v>
+      </c>
+      <c r="D59" s="9" t="s">
+        <v>39</v>
+      </c>
+      <c r="E59" s="7" t="s">
         <v>263</v>
       </c>
-      <c r="B59" s="9" t="s">
+      <c r="F59" s="9" t="s">
+        <v>260</v>
+      </c>
+      <c r="G59" s="7" t="s">
         <v>264</v>
       </c>
-      <c r="C59" s="9" t="s">
+      <c r="H59" s="7" t="s">
         <v>265</v>
-      </c>
-      <c r="D59" s="9" t="s">
-        <v>39</v>
-      </c>
-      <c r="E59" s="7" t="s">
-        <v>266</v>
-      </c>
-      <c r="F59" s="9" t="s">
-        <v>263</v>
-      </c>
-      <c r="G59" s="7" t="s">
-        <v>267</v>
-      </c>
-      <c r="H59" s="7" t="s">
-        <v>268</v>
       </c>
     </row>
     <row r="60" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -2979,6 +2962,7 @@
     <hyperlink ref="A41" r:id="rId2" display="katherine.salas.kniland@una.cr"/>
     <hyperlink ref="A42" r:id="rId3" display="katherine.salas.kniland@una.cr"/>
     <hyperlink ref="H47" r:id="rId4" display="karla.ramirez.amador@una.cr"/>
+    <hyperlink ref="H52" r:id="rId5" display="monica.narvaez.ruano@una.cr"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
@@ -2988,7 +2972,7 @@
     <oddFooter/>
   </headerFooter>
   <tableParts>
-    <tablePart r:id="rId5"/>
+    <tablePart r:id="rId6"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>